<commit_message>
Kalkylpris 2 på resursen
work_centers.calc_rate_2 (0162) som Kalkylpris 1: fält i resursformuläret, resursimportens "Aktuell, K.pris 2" mappas automatiskt, sparas som förvalsvärde som kalkylen ännu inte läser. Manual och importmall uppdaterade.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pvWaFZiioxpDd9AVeYPCR
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-resurser.xlsx
+++ b/apps/web/public/importmallar/importmall-resurser.xlsx
@@ -106,11 +106,23 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">Ett andra alternativt timpris i SEK, decimalkomma eller punkt, aldrig negativt. Sparas på resursen men används inte av kalkylen ännu.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — om timkostnaden gäller ställtiden. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="0">
+    <comment ref="J1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -122,7 +134,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="0">
+    <comment ref="K1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -134,7 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="0">
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -146,7 +158,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="0">
+    <comment ref="M1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -227,9 +239,10 @@
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="20" customWidth="1"/>
-    <col min="11" max="11" width="31" customWidth="1"/>
-    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="31" customWidth="1"/>
+    <col min="13" max="13" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -270,25 +283,30 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Kalkylpris 2</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Gäller ställ</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Gäller styck</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Förvald ställtid</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Förvald operationsbenämning</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Kostnadsrad</t>
         </is>
@@ -525,7 +543,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gäller ställ</t>
+          <t xml:space="preserve">Kalkylpris 2</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -535,19 +553,19 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — om timkostnaden gäller ställtiden. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ett andra alternativt timpris i SEK, decimalkomma eller punkt, aldrig negativt. Sparas på resursen men används inte av kalkylen ännu.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja</t>
+          <t xml:space="preserve">600</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gäller styck</t>
+          <t xml:space="preserve">Gäller ställ</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -557,7 +575,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — om timkostnaden gäller stycktiden. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — om timkostnaden gäller ställtiden. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -569,7 +587,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Förvald ställtid</t>
+          <t xml:space="preserve">Gäller styck</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -579,19 +597,19 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ställtid i minuter, decimalkomma eller punkt, aldrig negativ. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — om timkostnaden gäller stycktiden. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">Ja</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Förvald operationsbenämning</t>
+          <t xml:space="preserve">Förvald ställtid</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -601,32 +619,54 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operationsnamn, max 100 tecken. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ställtid i minuter, decimalkomma eller punkt, aldrig negativ. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laserskärning</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Förvald operationsbenämning</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Operationsnamn, max 100 tecken. Sparas på resursen som förvalsvärde; används inte av beredningen eller kalkylen ännu. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laserskärning</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Kostnadsrad</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nej</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Styrkolumn för filer med flera kostnadsrader per resurs: bara raden vars värde börjar med Ordinarie importeras; saknar resursen en sådan tas dess första rad med en varning. Lagras inte — ta bort kolumnen när filen har en rad per resurs.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Ordinarie</t>
         </is>

</xml_diff>